<commit_message>
Add country column to job application tracker
Include Ülke for each application and country breakdown on the Özet sheet.

Co-authored-by: nurpercn <nurpercn@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/Basvuru_Takip_Listesi.xlsx
+++ b/Basvuru_Takip_Listesi.xlsx
@@ -11,7 +11,7 @@
     <sheet name="Özet" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Başvurular'!$A$1:$I$41</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Başvurular'!$A$1:$J$41</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -50,7 +50,7 @@
       <b val="1"/>
     </font>
   </fonts>
-  <fills count="6">
+  <fills count="7">
     <fill>
       <patternFill/>
     </fill>
@@ -60,6 +60,11 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="001F4E79"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00DDEBF7"/>
       </patternFill>
     </fill>
     <fill>
@@ -104,7 +109,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="11">
+  <cellXfs count="12">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -115,16 +120,19 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="165" fontId="2" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="165" fontId="2" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="2" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="2" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -495,18 +503,19 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I41"/>
+  <dimension ref="A1:J41"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
     <col width="62" customWidth="1" min="2" max="2"/>
     <col width="38" customWidth="1" min="3" max="3"/>
     <col width="32" customWidth="1" min="4" max="4"/>
-    <col width="14" customWidth="1" min="5" max="5"/>
-    <col width="15" customWidth="1" min="6" max="6"/>
-    <col width="32" customWidth="1" min="7" max="7"/>
-    <col width="14" customWidth="1" min="8" max="8"/>
-    <col width="30" customWidth="1" min="9" max="9"/>
+    <col width="22" customWidth="1" min="5" max="5"/>
+    <col width="14" customWidth="1" min="6" max="6"/>
+    <col width="15" customWidth="1" min="7" max="7"/>
+    <col width="32" customWidth="1" min="8" max="8"/>
+    <col width="14" customWidth="1" min="9" max="9"/>
+    <col width="30" customWidth="1" min="10" max="10"/>
   </cols>
   <sheetData>
     <row r="1" ht="24" customHeight="1">
@@ -532,25 +541,30 @@
       </c>
       <c r="E1" s="1" t="inlineStr">
         <is>
+          <t>Ülke</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
           <t>Çalışma Şekli</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>Başvuru Tarihi</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>Durum</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>Geri Dönüş</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="J1" s="1" t="inlineStr">
         <is>
           <t>Notlar</t>
         </is>
@@ -575,56 +589,66 @@
           <t>Kungsbacka</t>
         </is>
       </c>
-      <c r="E2" s="3" t="inlineStr">
+      <c r="E2" s="4" t="inlineStr">
+        <is>
+          <t>İsveç</t>
+        </is>
+      </c>
+      <c r="F2" s="3" t="inlineStr">
         <is>
           <t>On-site</t>
         </is>
       </c>
-      <c r="F2" s="4" t="n">
+      <c r="G2" s="5" t="n">
         <v>46245</v>
       </c>
-      <c r="G2" s="3" t="inlineStr">
-        <is>
-          <t>Beklemede</t>
-        </is>
-      </c>
-      <c r="H2" s="3" t="inlineStr"/>
+      <c r="H2" s="3" t="inlineStr">
+        <is>
+          <t>Beklemede</t>
+        </is>
+      </c>
       <c r="I2" s="3" t="inlineStr"/>
+      <c r="J2" s="3" t="inlineStr"/>
     </row>
     <row r="3">
-      <c r="A3" s="5" t="n">
+      <c r="A3" s="6" t="n">
         <v>2</v>
       </c>
-      <c r="B3" s="6" t="inlineStr">
+      <c r="B3" s="7" t="inlineStr">
         <is>
           <t>Product Certification Manager m|w|d</t>
         </is>
       </c>
-      <c r="C3" s="6" t="inlineStr">
+      <c r="C3" s="7" t="inlineStr">
         <is>
           <t>Balluff EMEA</t>
         </is>
       </c>
-      <c r="D3" s="6" t="inlineStr">
+      <c r="D3" s="7" t="inlineStr">
         <is>
           <t>Neuhausen auf den Fildern</t>
         </is>
       </c>
-      <c r="E3" s="6" t="inlineStr">
+      <c r="E3" s="4" t="inlineStr">
+        <is>
+          <t>Almanya</t>
+        </is>
+      </c>
+      <c r="F3" s="7" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="F3" s="4" t="n">
+      <c r="G3" s="5" t="n">
         <v>46245</v>
       </c>
-      <c r="G3" s="6" t="inlineStr">
-        <is>
-          <t>Beklemede</t>
-        </is>
-      </c>
-      <c r="H3" s="6" t="inlineStr"/>
-      <c r="I3" s="6" t="inlineStr"/>
+      <c r="H3" s="7" t="inlineStr">
+        <is>
+          <t>Beklemede</t>
+        </is>
+      </c>
+      <c r="I3" s="7" t="inlineStr"/>
+      <c r="J3" s="7" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" s="2" t="n">
@@ -645,56 +669,66 @@
           <t>Bury St Edmunds</t>
         </is>
       </c>
-      <c r="E4" s="3" t="inlineStr">
+      <c r="E4" s="4" t="inlineStr">
+        <is>
+          <t>Birleşik Krallık</t>
+        </is>
+      </c>
+      <c r="F4" s="3" t="inlineStr">
         <is>
           <t>On-site</t>
         </is>
       </c>
-      <c r="F4" s="4" t="n">
+      <c r="G4" s="5" t="n">
         <v>46245</v>
       </c>
-      <c r="G4" s="3" t="inlineStr">
-        <is>
-          <t>Beklemede</t>
-        </is>
-      </c>
-      <c r="H4" s="3" t="inlineStr"/>
+      <c r="H4" s="3" t="inlineStr">
+        <is>
+          <t>Beklemede</t>
+        </is>
+      </c>
       <c r="I4" s="3" t="inlineStr"/>
+      <c r="J4" s="3" t="inlineStr"/>
     </row>
     <row r="5">
-      <c r="A5" s="5" t="n">
+      <c r="A5" s="6" t="n">
         <v>4</v>
       </c>
-      <c r="B5" s="6" t="inlineStr">
+      <c r="B5" s="7" t="inlineStr">
         <is>
           <t>Head of Product Compliance | CE, Product Safety &amp; EU Regulatory Compliance</t>
         </is>
       </c>
-      <c r="C5" s="6" t="inlineStr">
+      <c r="C5" s="7" t="inlineStr">
         <is>
           <t>Avance</t>
         </is>
       </c>
-      <c r="D5" s="6" t="inlineStr">
+      <c r="D5" s="7" t="inlineStr">
         <is>
           <t>Kerkrade</t>
         </is>
       </c>
-      <c r="E5" s="6" t="inlineStr">
+      <c r="E5" s="4" t="inlineStr">
+        <is>
+          <t>Hollanda</t>
+        </is>
+      </c>
+      <c r="F5" s="7" t="inlineStr">
         <is>
           <t>On-site</t>
         </is>
       </c>
-      <c r="F5" s="4" t="n">
+      <c r="G5" s="5" t="n">
         <v>46245</v>
       </c>
-      <c r="G5" s="6" t="inlineStr">
-        <is>
-          <t>Beklemede</t>
-        </is>
-      </c>
-      <c r="H5" s="6" t="inlineStr"/>
-      <c r="I5" s="6" t="inlineStr"/>
+      <c r="H5" s="7" t="inlineStr">
+        <is>
+          <t>Beklemede</t>
+        </is>
+      </c>
+      <c r="I5" s="7" t="inlineStr"/>
+      <c r="J5" s="7" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" s="2" t="n">
@@ -715,56 +749,66 @@
           <t>North Lincolnshire</t>
         </is>
       </c>
-      <c r="E6" s="3" t="inlineStr">
+      <c r="E6" s="4" t="inlineStr">
+        <is>
+          <t>Birleşik Krallık</t>
+        </is>
+      </c>
+      <c r="F6" s="3" t="inlineStr">
         <is>
           <t>On-site</t>
         </is>
       </c>
-      <c r="F6" s="4" t="n">
+      <c r="G6" s="5" t="n">
         <v>46245</v>
       </c>
-      <c r="G6" s="3" t="inlineStr">
-        <is>
-          <t>Beklemede</t>
-        </is>
-      </c>
-      <c r="H6" s="3" t="inlineStr"/>
+      <c r="H6" s="3" t="inlineStr">
+        <is>
+          <t>Beklemede</t>
+        </is>
+      </c>
       <c r="I6" s="3" t="inlineStr"/>
+      <c r="J6" s="3" t="inlineStr"/>
     </row>
     <row r="7">
-      <c r="A7" s="5" t="n">
+      <c r="A7" s="6" t="n">
         <v>6</v>
       </c>
-      <c r="B7" s="6" t="inlineStr">
+      <c r="B7" s="7" t="inlineStr">
         <is>
           <t>Regulatory Affairs Manager - New Countries</t>
         </is>
       </c>
-      <c r="C7" s="6" t="inlineStr">
+      <c r="C7" s="7" t="inlineStr">
         <is>
           <t>Action</t>
         </is>
       </c>
-      <c r="D7" s="6" t="inlineStr">
+      <c r="D7" s="7" t="inlineStr">
         <is>
           <t>Zwaagdijk-Oost</t>
         </is>
       </c>
-      <c r="E7" s="6" t="inlineStr">
+      <c r="E7" s="4" t="inlineStr">
+        <is>
+          <t>Hollanda</t>
+        </is>
+      </c>
+      <c r="F7" s="7" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="F7" s="4" t="n">
+      <c r="G7" s="5" t="n">
         <v>46245</v>
       </c>
-      <c r="G7" s="6" t="inlineStr">
-        <is>
-          <t>Beklemede</t>
-        </is>
-      </c>
-      <c r="H7" s="6" t="inlineStr"/>
-      <c r="I7" s="6" t="inlineStr"/>
+      <c r="H7" s="7" t="inlineStr">
+        <is>
+          <t>Beklemede</t>
+        </is>
+      </c>
+      <c r="I7" s="7" t="inlineStr"/>
+      <c r="J7" s="7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" s="2" t="n">
@@ -785,56 +829,66 @@
           <t>Nottingham</t>
         </is>
       </c>
-      <c r="E8" s="3" t="inlineStr">
+      <c r="E8" s="4" t="inlineStr">
+        <is>
+          <t>Birleşik Krallık</t>
+        </is>
+      </c>
+      <c r="F8" s="3" t="inlineStr">
         <is>
           <t>Hybrid</t>
         </is>
       </c>
-      <c r="F8" s="4" t="n">
+      <c r="G8" s="5" t="n">
         <v>46245</v>
       </c>
-      <c r="G8" s="3" t="inlineStr">
-        <is>
-          <t>Beklemede</t>
-        </is>
-      </c>
-      <c r="H8" s="3" t="inlineStr"/>
+      <c r="H8" s="3" t="inlineStr">
+        <is>
+          <t>Beklemede</t>
+        </is>
+      </c>
       <c r="I8" s="3" t="inlineStr"/>
+      <c r="J8" s="3" t="inlineStr"/>
     </row>
     <row r="9">
-      <c r="A9" s="5" t="n">
+      <c r="A9" s="6" t="n">
         <v>8</v>
       </c>
-      <c r="B9" s="6" t="inlineStr">
+      <c r="B9" s="7" t="inlineStr">
         <is>
           <t>Product Compliance Lead</t>
         </is>
       </c>
-      <c r="C9" s="6" t="inlineStr">
+      <c r="C9" s="7" t="inlineStr">
         <is>
           <t>MUJI Finland Oy</t>
         </is>
       </c>
-      <c r="D9" s="6" t="inlineStr">
+      <c r="D9" s="7" t="inlineStr">
         <is>
           <t>London</t>
         </is>
       </c>
-      <c r="E9" s="6" t="inlineStr">
+      <c r="E9" s="4" t="inlineStr">
+        <is>
+          <t>Birleşik Krallık</t>
+        </is>
+      </c>
+      <c r="F9" s="7" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="F9" s="4" t="n">
+      <c r="G9" s="5" t="n">
         <v>46245</v>
       </c>
-      <c r="G9" s="6" t="inlineStr">
-        <is>
-          <t>Beklemede</t>
-        </is>
-      </c>
-      <c r="H9" s="6" t="inlineStr"/>
-      <c r="I9" s="6" t="inlineStr"/>
+      <c r="H9" s="7" t="inlineStr">
+        <is>
+          <t>Beklemede</t>
+        </is>
+      </c>
+      <c r="I9" s="7" t="inlineStr"/>
+      <c r="J9" s="7" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" s="2" t="n">
@@ -855,56 +909,66 @@
           <t>London Area, United Kingdom</t>
         </is>
       </c>
-      <c r="E10" s="3" t="inlineStr">
+      <c r="E10" s="4" t="inlineStr">
+        <is>
+          <t>Birleşik Krallık</t>
+        </is>
+      </c>
+      <c r="F10" s="3" t="inlineStr">
         <is>
           <t>On-site</t>
         </is>
       </c>
-      <c r="F10" s="4" t="n">
+      <c r="G10" s="5" t="n">
         <v>46245</v>
       </c>
-      <c r="G10" s="3" t="inlineStr">
-        <is>
-          <t>Beklemede</t>
-        </is>
-      </c>
-      <c r="H10" s="3" t="inlineStr"/>
+      <c r="H10" s="3" t="inlineStr">
+        <is>
+          <t>Beklemede</t>
+        </is>
+      </c>
       <c r="I10" s="3" t="inlineStr"/>
+      <c r="J10" s="3" t="inlineStr"/>
     </row>
     <row r="11">
-      <c r="A11" s="5" t="n">
+      <c r="A11" s="6" t="n">
         <v>10</v>
       </c>
-      <c r="B11" s="6" t="inlineStr">
+      <c r="B11" s="7" t="inlineStr">
         <is>
           <t>Regulatory Affairs Specialist</t>
         </is>
       </c>
-      <c r="C11" s="6" t="inlineStr">
+      <c r="C11" s="7" t="inlineStr">
         <is>
           <t>Cranleigh STEM &amp; Sustainability Recruitment</t>
         </is>
       </c>
-      <c r="D11" s="6" t="inlineStr">
+      <c r="D11" s="7" t="inlineStr">
         <is>
           <t>Carlisle</t>
         </is>
       </c>
-      <c r="E11" s="6" t="inlineStr">
+      <c r="E11" s="4" t="inlineStr">
+        <is>
+          <t>Birleşik Krallık</t>
+        </is>
+      </c>
+      <c r="F11" s="7" t="inlineStr">
         <is>
           <t>Hybrid</t>
         </is>
       </c>
-      <c r="F11" s="4" t="n">
+      <c r="G11" s="5" t="n">
         <v>46245</v>
       </c>
-      <c r="G11" s="6" t="inlineStr">
-        <is>
-          <t>Beklemede</t>
-        </is>
-      </c>
-      <c r="H11" s="6" t="inlineStr"/>
-      <c r="I11" s="6" t="inlineStr"/>
+      <c r="H11" s="7" t="inlineStr">
+        <is>
+          <t>Beklemede</t>
+        </is>
+      </c>
+      <c r="I11" s="7" t="inlineStr"/>
+      <c r="J11" s="7" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" s="2" t="n">
@@ -925,56 +989,66 @@
           <t>Oldbury</t>
         </is>
       </c>
-      <c r="E12" s="3" t="inlineStr">
+      <c r="E12" s="4" t="inlineStr">
+        <is>
+          <t>Birleşik Krallık</t>
+        </is>
+      </c>
+      <c r="F12" s="3" t="inlineStr">
         <is>
           <t>On-site</t>
         </is>
       </c>
-      <c r="F12" s="4" t="n">
+      <c r="G12" s="5" t="n">
         <v>46245</v>
       </c>
-      <c r="G12" s="3" t="inlineStr">
-        <is>
-          <t>Beklemede</t>
-        </is>
-      </c>
-      <c r="H12" s="3" t="inlineStr"/>
+      <c r="H12" s="3" t="inlineStr">
+        <is>
+          <t>Beklemede</t>
+        </is>
+      </c>
       <c r="I12" s="3" t="inlineStr"/>
+      <c r="J12" s="3" t="inlineStr"/>
     </row>
     <row r="13">
-      <c r="A13" s="5" t="n">
+      <c r="A13" s="6" t="n">
         <v>12</v>
       </c>
-      <c r="B13" s="6" t="inlineStr">
+      <c r="B13" s="7" t="inlineStr">
         <is>
           <t>Technical Compliance &amp; Certification Officer</t>
         </is>
       </c>
-      <c r="C13" s="6" t="inlineStr">
+      <c r="C13" s="7" t="inlineStr">
         <is>
           <t>Solutions Driven</t>
         </is>
       </c>
-      <c r="D13" s="6" t="inlineStr">
+      <c r="D13" s="7" t="inlineStr">
         <is>
           <t>Portishead</t>
         </is>
       </c>
-      <c r="E13" s="6" t="inlineStr">
+      <c r="E13" s="4" t="inlineStr">
+        <is>
+          <t>Birleşik Krallık</t>
+        </is>
+      </c>
+      <c r="F13" s="7" t="inlineStr">
         <is>
           <t>Hybrid</t>
         </is>
       </c>
-      <c r="F13" s="4" t="n">
+      <c r="G13" s="5" t="n">
         <v>46245</v>
       </c>
-      <c r="G13" s="6" t="inlineStr">
-        <is>
-          <t>Beklemede</t>
-        </is>
-      </c>
-      <c r="H13" s="6" t="inlineStr"/>
-      <c r="I13" s="6" t="inlineStr"/>
+      <c r="H13" s="7" t="inlineStr">
+        <is>
+          <t>Beklemede</t>
+        </is>
+      </c>
+      <c r="I13" s="7" t="inlineStr"/>
+      <c r="J13" s="7" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" s="2" t="n">
@@ -995,56 +1069,66 @@
           <t>Bradford</t>
         </is>
       </c>
-      <c r="E14" s="3" t="inlineStr">
+      <c r="E14" s="4" t="inlineStr">
+        <is>
+          <t>Birleşik Krallık</t>
+        </is>
+      </c>
+      <c r="F14" s="3" t="inlineStr">
         <is>
           <t>On-site</t>
         </is>
       </c>
-      <c r="F14" s="4" t="n">
+      <c r="G14" s="5" t="n">
         <v>46243</v>
       </c>
-      <c r="G14" s="3" t="inlineStr">
-        <is>
-          <t>Beklemede</t>
-        </is>
-      </c>
-      <c r="H14" s="3" t="inlineStr"/>
+      <c r="H14" s="3" t="inlineStr">
+        <is>
+          <t>Beklemede</t>
+        </is>
+      </c>
       <c r="I14" s="3" t="inlineStr"/>
+      <c r="J14" s="3" t="inlineStr"/>
     </row>
     <row r="15">
-      <c r="A15" s="5" t="n">
+      <c r="A15" s="6" t="n">
         <v>14</v>
       </c>
-      <c r="B15" s="6" t="inlineStr">
+      <c r="B15" s="7" t="inlineStr">
         <is>
           <t>Product Compliance Engineer</t>
         </is>
       </c>
-      <c r="C15" s="6" t="inlineStr">
+      <c r="C15" s="7" t="inlineStr">
         <is>
           <t>Platform Recruitment</t>
         </is>
       </c>
-      <c r="D15" s="6" t="inlineStr">
+      <c r="D15" s="7" t="inlineStr">
         <is>
           <t>Bury St Edmunds</t>
         </is>
       </c>
-      <c r="E15" s="6" t="inlineStr">
+      <c r="E15" s="4" t="inlineStr">
+        <is>
+          <t>Birleşik Krallık</t>
+        </is>
+      </c>
+      <c r="F15" s="7" t="inlineStr">
         <is>
           <t>On-site</t>
         </is>
       </c>
-      <c r="F15" s="4" t="n">
+      <c r="G15" s="5" t="n">
         <v>46243</v>
       </c>
-      <c r="G15" s="7" t="inlineStr">
+      <c r="H15" s="8" t="inlineStr">
         <is>
           <t>No longer accepting applications</t>
         </is>
       </c>
-      <c r="H15" s="6" t="inlineStr"/>
-      <c r="I15" s="6" t="inlineStr"/>
+      <c r="I15" s="7" t="inlineStr"/>
+      <c r="J15" s="7" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" s="2" t="n">
@@ -1065,56 +1149,66 @@
           <t>Oldham</t>
         </is>
       </c>
-      <c r="E16" s="3" t="inlineStr">
+      <c r="E16" s="4" t="inlineStr">
+        <is>
+          <t>Birleşik Krallık</t>
+        </is>
+      </c>
+      <c r="F16" s="3" t="inlineStr">
         <is>
           <t>Hybrid</t>
         </is>
       </c>
-      <c r="F16" s="4" t="n">
+      <c r="G16" s="5" t="n">
         <v>46243</v>
       </c>
-      <c r="G16" s="3" t="inlineStr">
-        <is>
-          <t>Beklemede</t>
-        </is>
-      </c>
-      <c r="H16" s="3" t="inlineStr"/>
+      <c r="H16" s="3" t="inlineStr">
+        <is>
+          <t>Beklemede</t>
+        </is>
+      </c>
       <c r="I16" s="3" t="inlineStr"/>
+      <c r="J16" s="3" t="inlineStr"/>
     </row>
     <row r="17">
-      <c r="A17" s="5" t="n">
+      <c r="A17" s="6" t="n">
         <v>16</v>
       </c>
-      <c r="B17" s="6" t="inlineStr">
+      <c r="B17" s="7" t="inlineStr">
         <is>
           <t>Product Certification Engineer</t>
         </is>
       </c>
-      <c r="C17" s="6" t="inlineStr">
+      <c r="C17" s="7" t="inlineStr">
         <is>
           <t>Omega</t>
         </is>
       </c>
-      <c r="D17" s="6" t="inlineStr">
+      <c r="D17" s="7" t="inlineStr">
         <is>
           <t>Stroud</t>
         </is>
       </c>
-      <c r="E17" s="6" t="inlineStr">
+      <c r="E17" s="4" t="inlineStr">
+        <is>
+          <t>Birleşik Krallık</t>
+        </is>
+      </c>
+      <c r="F17" s="7" t="inlineStr">
         <is>
           <t>Hybrid</t>
         </is>
       </c>
-      <c r="F17" s="4" t="n">
+      <c r="G17" s="5" t="n">
         <v>46243</v>
       </c>
-      <c r="G17" s="6" t="inlineStr">
-        <is>
-          <t>Beklemede</t>
-        </is>
-      </c>
-      <c r="H17" s="6" t="inlineStr"/>
-      <c r="I17" s="6" t="inlineStr"/>
+      <c r="H17" s="7" t="inlineStr">
+        <is>
+          <t>Beklemede</t>
+        </is>
+      </c>
+      <c r="I17" s="7" t="inlineStr"/>
+      <c r="J17" s="7" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" s="2" t="n">
@@ -1135,56 +1229,66 @@
           <t>Brussels</t>
         </is>
       </c>
-      <c r="E18" s="3" t="inlineStr">
+      <c r="E18" s="4" t="inlineStr">
+        <is>
+          <t>Belçika</t>
+        </is>
+      </c>
+      <c r="F18" s="3" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="F18" s="4" t="n">
+      <c r="G18" s="5" t="n">
         <v>46242</v>
       </c>
-      <c r="G18" s="3" t="inlineStr">
-        <is>
-          <t>Beklemede</t>
-        </is>
-      </c>
-      <c r="H18" s="3" t="inlineStr"/>
+      <c r="H18" s="3" t="inlineStr">
+        <is>
+          <t>Beklemede</t>
+        </is>
+      </c>
       <c r="I18" s="3" t="inlineStr"/>
+      <c r="J18" s="3" t="inlineStr"/>
     </row>
     <row r="19">
-      <c r="A19" s="5" t="n">
+      <c r="A19" s="6" t="n">
         <v>18</v>
       </c>
-      <c r="B19" s="6" t="inlineStr">
+      <c r="B19" s="7" t="inlineStr">
         <is>
           <t>Compliance Manager (Solar, Air Con &amp; EV Chargers)</t>
         </is>
       </c>
-      <c r="C19" s="6" t="inlineStr">
+      <c r="C19" s="7" t="inlineStr">
         <is>
           <t>R&amp;O Property Services LTD</t>
         </is>
       </c>
-      <c r="D19" s="6" t="inlineStr">
+      <c r="D19" s="7" t="inlineStr">
         <is>
           <t>Greater London</t>
         </is>
       </c>
-      <c r="E19" s="6" t="inlineStr">
+      <c r="E19" s="4" t="inlineStr">
+        <is>
+          <t>Birleşik Krallık</t>
+        </is>
+      </c>
+      <c r="F19" s="7" t="inlineStr">
         <is>
           <t>On-site</t>
         </is>
       </c>
-      <c r="F19" s="4" t="n">
+      <c r="G19" s="5" t="n">
         <v>46242</v>
       </c>
-      <c r="G19" s="6" t="inlineStr">
-        <is>
-          <t>Beklemede</t>
-        </is>
-      </c>
-      <c r="H19" s="6" t="inlineStr"/>
-      <c r="I19" s="6" t="inlineStr"/>
+      <c r="H19" s="7" t="inlineStr">
+        <is>
+          <t>Beklemede</t>
+        </is>
+      </c>
+      <c r="I19" s="7" t="inlineStr"/>
+      <c r="J19" s="7" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" s="2" t="n">
@@ -1205,56 +1309,66 @@
           <t>South Yorkshire</t>
         </is>
       </c>
-      <c r="E20" s="3" t="inlineStr">
+      <c r="E20" s="4" t="inlineStr">
+        <is>
+          <t>Birleşik Krallık</t>
+        </is>
+      </c>
+      <c r="F20" s="3" t="inlineStr">
         <is>
           <t>On-site</t>
         </is>
       </c>
-      <c r="F20" s="4" t="n">
+      <c r="G20" s="5" t="n">
         <v>46241</v>
       </c>
-      <c r="G20" s="3" t="inlineStr">
-        <is>
-          <t>Beklemede</t>
-        </is>
-      </c>
-      <c r="H20" s="3" t="inlineStr"/>
+      <c r="H20" s="3" t="inlineStr">
+        <is>
+          <t>Beklemede</t>
+        </is>
+      </c>
       <c r="I20" s="3" t="inlineStr"/>
+      <c r="J20" s="3" t="inlineStr"/>
     </row>
     <row r="21">
-      <c r="A21" s="5" t="n">
+      <c r="A21" s="6" t="n">
         <v>20</v>
       </c>
-      <c r="B21" s="6" t="inlineStr">
+      <c r="B21" s="7" t="inlineStr">
         <is>
           <t>Compliance Manager</t>
         </is>
       </c>
-      <c r="C21" s="6" t="inlineStr">
+      <c r="C21" s="7" t="inlineStr">
         <is>
           <t>KO2 Embedded Recruitment Solutions Ltd</t>
         </is>
       </c>
-      <c r="D21" s="6" t="inlineStr">
+      <c r="D21" s="7" t="inlineStr">
         <is>
           <t>Ormskirk</t>
         </is>
       </c>
-      <c r="E21" s="6" t="inlineStr">
+      <c r="E21" s="4" t="inlineStr">
+        <is>
+          <t>Birleşik Krallık</t>
+        </is>
+      </c>
+      <c r="F21" s="7" t="inlineStr">
         <is>
           <t>On-site</t>
         </is>
       </c>
-      <c r="F21" s="4" t="n">
+      <c r="G21" s="5" t="n">
         <v>46241</v>
       </c>
-      <c r="G21" s="6" t="inlineStr">
-        <is>
-          <t>Beklemede</t>
-        </is>
-      </c>
-      <c r="H21" s="6" t="inlineStr"/>
-      <c r="I21" s="6" t="inlineStr"/>
+      <c r="H21" s="7" t="inlineStr">
+        <is>
+          <t>Beklemede</t>
+        </is>
+      </c>
+      <c r="I21" s="7" t="inlineStr"/>
+      <c r="J21" s="7" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" s="2" t="n">
@@ -1275,56 +1389,66 @@
           <t>Manchester Area, United Kingdom</t>
         </is>
       </c>
-      <c r="E22" s="3" t="inlineStr">
+      <c r="E22" s="4" t="inlineStr">
+        <is>
+          <t>Birleşik Krallık</t>
+        </is>
+      </c>
+      <c r="F22" s="3" t="inlineStr">
         <is>
           <t>On-site</t>
         </is>
       </c>
-      <c r="F22" s="4" t="n">
+      <c r="G22" s="5" t="n">
         <v>46240</v>
       </c>
-      <c r="G22" s="3" t="inlineStr">
-        <is>
-          <t>Beklemede</t>
-        </is>
-      </c>
-      <c r="H22" s="3" t="inlineStr"/>
+      <c r="H22" s="3" t="inlineStr">
+        <is>
+          <t>Beklemede</t>
+        </is>
+      </c>
       <c r="I22" s="3" t="inlineStr"/>
+      <c r="J22" s="3" t="inlineStr"/>
     </row>
     <row r="23">
-      <c r="A23" s="5" t="n">
+      <c r="A23" s="6" t="n">
         <v>22</v>
       </c>
-      <c r="B23" s="6" t="inlineStr">
+      <c r="B23" s="7" t="inlineStr">
         <is>
           <t>Technical Compliance &amp; Certification Officer</t>
         </is>
       </c>
-      <c r="C23" s="6" t="inlineStr">
+      <c r="C23" s="7" t="inlineStr">
         <is>
           <t>Solutions Driven</t>
         </is>
       </c>
-      <c r="D23" s="6" t="inlineStr">
+      <c r="D23" s="7" t="inlineStr">
         <is>
           <t>Portishead</t>
         </is>
       </c>
-      <c r="E23" s="6" t="inlineStr">
+      <c r="E23" s="4" t="inlineStr">
+        <is>
+          <t>Birleşik Krallık</t>
+        </is>
+      </c>
+      <c r="F23" s="7" t="inlineStr">
         <is>
           <t>Hybrid</t>
         </is>
       </c>
-      <c r="F23" s="4" t="n">
+      <c r="G23" s="5" t="n">
         <v>46240</v>
       </c>
-      <c r="G23" s="7" t="inlineStr">
+      <c r="H23" s="8" t="inlineStr">
         <is>
           <t>No longer accepting applications</t>
         </is>
       </c>
-      <c r="H23" s="6" t="inlineStr"/>
-      <c r="I23" s="6" t="inlineStr"/>
+      <c r="I23" s="7" t="inlineStr"/>
+      <c r="J23" s="7" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" s="2" t="n">
@@ -1345,56 +1469,66 @@
           <t>Istanbul, Türkiye</t>
         </is>
       </c>
-      <c r="E24" s="3" t="inlineStr">
+      <c r="E24" s="4" t="inlineStr">
+        <is>
+          <t>Türkiye</t>
+        </is>
+      </c>
+      <c r="F24" s="3" t="inlineStr">
         <is>
           <t>On-site</t>
         </is>
       </c>
-      <c r="F24" s="4" t="n">
+      <c r="G24" s="5" t="n">
         <v>46239</v>
       </c>
-      <c r="G24" s="3" t="inlineStr">
-        <is>
-          <t>Beklemede</t>
-        </is>
-      </c>
-      <c r="H24" s="3" t="inlineStr"/>
+      <c r="H24" s="3" t="inlineStr">
+        <is>
+          <t>Beklemede</t>
+        </is>
+      </c>
       <c r="I24" s="3" t="inlineStr"/>
+      <c r="J24" s="3" t="inlineStr"/>
     </row>
     <row r="25">
-      <c r="A25" s="5" t="n">
+      <c r="A25" s="6" t="n">
         <v>24</v>
       </c>
-      <c r="B25" s="6" t="inlineStr">
+      <c r="B25" s="7" t="inlineStr">
         <is>
           <t>Product Safety Engineer</t>
         </is>
       </c>
-      <c r="C25" s="6" t="inlineStr">
+      <c r="C25" s="7" t="inlineStr">
         <is>
           <t>Bulgin</t>
         </is>
       </c>
-      <c r="D25" s="6" t="inlineStr">
+      <c r="D25" s="7" t="inlineStr">
         <is>
           <t>Cambridge</t>
         </is>
       </c>
-      <c r="E25" s="6" t="inlineStr">
+      <c r="E25" s="4" t="inlineStr">
+        <is>
+          <t>Birleşik Krallık</t>
+        </is>
+      </c>
+      <c r="F25" s="7" t="inlineStr">
         <is>
           <t>On-site</t>
         </is>
       </c>
-      <c r="F25" s="4" t="n">
+      <c r="G25" s="5" t="n">
         <v>46239</v>
       </c>
-      <c r="G25" s="7" t="inlineStr">
+      <c r="H25" s="8" t="inlineStr">
         <is>
           <t>No longer accepting applications</t>
         </is>
       </c>
-      <c r="H25" s="6" t="inlineStr"/>
-      <c r="I25" s="6" t="inlineStr"/>
+      <c r="I25" s="7" t="inlineStr"/>
+      <c r="J25" s="7" t="inlineStr"/>
     </row>
     <row r="26">
       <c r="A26" s="2" t="n">
@@ -1415,56 +1549,66 @@
           <t>England, United Kingdom</t>
         </is>
       </c>
-      <c r="E26" s="3" t="inlineStr">
+      <c r="E26" s="4" t="inlineStr">
+        <is>
+          <t>Birleşik Krallık</t>
+        </is>
+      </c>
+      <c r="F26" s="3" t="inlineStr">
         <is>
           <t>Remote</t>
         </is>
       </c>
-      <c r="F26" s="4" t="n">
+      <c r="G26" s="5" t="n">
         <v>46239</v>
       </c>
-      <c r="G26" s="7" t="inlineStr">
+      <c r="H26" s="8" t="inlineStr">
         <is>
           <t>No longer accepting applications</t>
         </is>
       </c>
-      <c r="H26" s="3" t="inlineStr"/>
       <c r="I26" s="3" t="inlineStr"/>
+      <c r="J26" s="3" t="inlineStr"/>
     </row>
     <row r="27">
-      <c r="A27" s="5" t="n">
+      <c r="A27" s="6" t="n">
         <v>26</v>
       </c>
-      <c r="B27" s="6" t="inlineStr">
+      <c r="B27" s="7" t="inlineStr">
         <is>
           <t>Export Control and Regulatory Coordinator</t>
         </is>
       </c>
-      <c r="C27" s="6" t="inlineStr">
+      <c r="C27" s="7" t="inlineStr">
         <is>
           <t>Luxfer MEL Technologies</t>
         </is>
       </c>
-      <c r="D27" s="6" t="inlineStr">
+      <c r="D27" s="7" t="inlineStr">
         <is>
           <t>Swinton</t>
         </is>
       </c>
-      <c r="E27" s="6" t="inlineStr">
+      <c r="E27" s="4" t="inlineStr">
+        <is>
+          <t>Birleşik Krallık</t>
+        </is>
+      </c>
+      <c r="F27" s="7" t="inlineStr">
         <is>
           <t>On-site</t>
         </is>
       </c>
-      <c r="F27" s="4" t="n">
+      <c r="G27" s="5" t="n">
         <v>46239</v>
       </c>
-      <c r="G27" s="6" t="inlineStr">
-        <is>
-          <t>Beklemede</t>
-        </is>
-      </c>
-      <c r="H27" s="6" t="inlineStr"/>
-      <c r="I27" s="6" t="inlineStr"/>
+      <c r="H27" s="7" t="inlineStr">
+        <is>
+          <t>Beklemede</t>
+        </is>
+      </c>
+      <c r="I27" s="7" t="inlineStr"/>
+      <c r="J27" s="7" t="inlineStr"/>
     </row>
     <row r="28">
       <c r="A28" s="2" t="n">
@@ -1485,56 +1629,66 @@
           <t>England, United Kingdom</t>
         </is>
       </c>
-      <c r="E28" s="3" t="inlineStr">
+      <c r="E28" s="4" t="inlineStr">
+        <is>
+          <t>Birleşik Krallık</t>
+        </is>
+      </c>
+      <c r="F28" s="3" t="inlineStr">
         <is>
           <t>On-site</t>
         </is>
       </c>
-      <c r="F28" s="4" t="n">
+      <c r="G28" s="5" t="n">
         <v>46239</v>
       </c>
-      <c r="G28" s="3" t="inlineStr">
-        <is>
-          <t>Beklemede</t>
-        </is>
-      </c>
-      <c r="H28" s="3" t="inlineStr"/>
+      <c r="H28" s="3" t="inlineStr">
+        <is>
+          <t>Beklemede</t>
+        </is>
+      </c>
       <c r="I28" s="3" t="inlineStr"/>
+      <c r="J28" s="3" t="inlineStr"/>
     </row>
     <row r="29">
-      <c r="A29" s="5" t="n">
+      <c r="A29" s="6" t="n">
         <v>28</v>
       </c>
-      <c r="B29" s="6" t="inlineStr">
+      <c r="B29" s="7" t="inlineStr">
         <is>
           <t>Technical Manager (INFORMED Certification Programs)</t>
         </is>
       </c>
-      <c r="C29" s="6" t="inlineStr">
+      <c r="C29" s="7" t="inlineStr">
         <is>
           <t>LGC, Biosearch Technologies</t>
         </is>
       </c>
-      <c r="D29" s="6" t="inlineStr">
+      <c r="D29" s="7" t="inlineStr">
         <is>
           <t>Cambridge</t>
         </is>
       </c>
-      <c r="E29" s="6" t="inlineStr">
+      <c r="E29" s="4" t="inlineStr">
+        <is>
+          <t>Birleşik Krallık</t>
+        </is>
+      </c>
+      <c r="F29" s="7" t="inlineStr">
         <is>
           <t>Remote</t>
         </is>
       </c>
-      <c r="F29" s="4" t="n">
+      <c r="G29" s="5" t="n">
         <v>46239</v>
       </c>
-      <c r="G29" s="6" t="inlineStr">
-        <is>
-          <t>Beklemede</t>
-        </is>
-      </c>
-      <c r="H29" s="6" t="inlineStr"/>
-      <c r="I29" s="6" t="inlineStr"/>
+      <c r="H29" s="7" t="inlineStr">
+        <is>
+          <t>Beklemede</t>
+        </is>
+      </c>
+      <c r="I29" s="7" t="inlineStr"/>
+      <c r="J29" s="7" t="inlineStr"/>
     </row>
     <row r="30">
       <c r="A30" s="2" t="n">
@@ -1555,56 +1709,66 @@
           <t>Istanbul, Türkiye</t>
         </is>
       </c>
-      <c r="E30" s="3" t="inlineStr">
+      <c r="E30" s="4" t="inlineStr">
+        <is>
+          <t>Türkiye</t>
+        </is>
+      </c>
+      <c r="F30" s="3" t="inlineStr">
         <is>
           <t>Remote</t>
         </is>
       </c>
-      <c r="F30" s="4" t="n">
+      <c r="G30" s="5" t="n">
         <v>46239</v>
       </c>
-      <c r="G30" s="3" t="inlineStr">
-        <is>
-          <t>Beklemede</t>
-        </is>
-      </c>
-      <c r="H30" s="3" t="inlineStr"/>
+      <c r="H30" s="3" t="inlineStr">
+        <is>
+          <t>Beklemede</t>
+        </is>
+      </c>
       <c r="I30" s="3" t="inlineStr"/>
+      <c r="J30" s="3" t="inlineStr"/>
     </row>
     <row r="31">
-      <c r="A31" s="5" t="n">
+      <c r="A31" s="6" t="n">
         <v>30</v>
       </c>
-      <c r="B31" s="6" t="inlineStr">
+      <c r="B31" s="7" t="inlineStr">
         <is>
           <t>Global Regulation Specialist</t>
         </is>
       </c>
-      <c r="C31" s="6" t="inlineStr">
+      <c r="C31" s="7" t="inlineStr">
         <is>
           <t>Hayat Kimya</t>
         </is>
       </c>
-      <c r="D31" s="6" t="inlineStr">
+      <c r="D31" s="7" t="inlineStr">
         <is>
           <t>Istanbul, Türkiye</t>
         </is>
       </c>
-      <c r="E31" s="6" t="inlineStr">
+      <c r="E31" s="4" t="inlineStr">
+        <is>
+          <t>Türkiye</t>
+        </is>
+      </c>
+      <c r="F31" s="7" t="inlineStr">
         <is>
           <t>Hybrid</t>
         </is>
       </c>
-      <c r="F31" s="4" t="n">
+      <c r="G31" s="5" t="n">
         <v>46239</v>
       </c>
-      <c r="G31" s="6" t="inlineStr">
-        <is>
-          <t>Beklemede</t>
-        </is>
-      </c>
-      <c r="H31" s="6" t="inlineStr"/>
-      <c r="I31" s="6" t="inlineStr"/>
+      <c r="H31" s="7" t="inlineStr">
+        <is>
+          <t>Beklemede</t>
+        </is>
+      </c>
+      <c r="I31" s="7" t="inlineStr"/>
+      <c r="J31" s="7" t="inlineStr"/>
     </row>
     <row r="32">
       <c r="A32" s="2" t="n">
@@ -1625,56 +1789,66 @@
           <t>Greater Leeds Area</t>
         </is>
       </c>
-      <c r="E32" s="3" t="inlineStr">
+      <c r="E32" s="4" t="inlineStr">
+        <is>
+          <t>Birleşik Krallık</t>
+        </is>
+      </c>
+      <c r="F32" s="3" t="inlineStr">
         <is>
           <t>Hybrid</t>
         </is>
       </c>
-      <c r="F32" s="4" t="n">
+      <c r="G32" s="5" t="n">
         <v>46239</v>
       </c>
-      <c r="G32" s="3" t="inlineStr">
-        <is>
-          <t>Beklemede</t>
-        </is>
-      </c>
-      <c r="H32" s="3" t="inlineStr"/>
+      <c r="H32" s="3" t="inlineStr">
+        <is>
+          <t>Beklemede</t>
+        </is>
+      </c>
       <c r="I32" s="3" t="inlineStr"/>
+      <c r="J32" s="3" t="inlineStr"/>
     </row>
     <row r="33">
-      <c r="A33" s="5" t="n">
+      <c r="A33" s="6" t="n">
         <v>32</v>
       </c>
-      <c r="B33" s="6" t="inlineStr">
+      <c r="B33" s="7" t="inlineStr">
         <is>
           <t>Head of Product Quality and Compliance</t>
         </is>
       </c>
-      <c r="C33" s="6" t="inlineStr">
+      <c r="C33" s="7" t="inlineStr">
         <is>
           <t>Pod Talent</t>
         </is>
       </c>
-      <c r="D33" s="6" t="inlineStr">
+      <c r="D33" s="7" t="inlineStr">
         <is>
           <t>Scotland, United Kingdom</t>
         </is>
       </c>
-      <c r="E33" s="6" t="inlineStr">
+      <c r="E33" s="4" t="inlineStr">
+        <is>
+          <t>Birleşik Krallık</t>
+        </is>
+      </c>
+      <c r="F33" s="7" t="inlineStr">
         <is>
           <t>On-site</t>
         </is>
       </c>
-      <c r="F33" s="4" t="n">
+      <c r="G33" s="5" t="n">
         <v>46239</v>
       </c>
-      <c r="G33" s="7" t="inlineStr">
+      <c r="H33" s="8" t="inlineStr">
         <is>
           <t>No longer accepting applications</t>
         </is>
       </c>
-      <c r="H33" s="6" t="inlineStr"/>
-      <c r="I33" s="6" t="inlineStr"/>
+      <c r="I33" s="7" t="inlineStr"/>
+      <c r="J33" s="7" t="inlineStr"/>
     </row>
     <row r="34">
       <c r="A34" s="2" t="n">
@@ -1695,56 +1869,66 @@
           <t>Biandronno</t>
         </is>
       </c>
-      <c r="E34" s="3" t="inlineStr">
+      <c r="E34" s="4" t="inlineStr">
+        <is>
+          <t>İtalya</t>
+        </is>
+      </c>
+      <c r="F34" s="3" t="inlineStr">
         <is>
           <t>On-site</t>
         </is>
       </c>
-      <c r="F34" s="4" t="n">
+      <c r="G34" s="5" t="n">
         <v>46239</v>
       </c>
-      <c r="G34" s="3" t="inlineStr">
-        <is>
-          <t>Beklemede</t>
-        </is>
-      </c>
-      <c r="H34" s="3" t="inlineStr"/>
+      <c r="H34" s="3" t="inlineStr">
+        <is>
+          <t>Beklemede</t>
+        </is>
+      </c>
       <c r="I34" s="3" t="inlineStr"/>
+      <c r="J34" s="3" t="inlineStr"/>
     </row>
     <row r="35">
-      <c r="A35" s="5" t="n">
+      <c r="A35" s="6" t="n">
         <v>34</v>
       </c>
-      <c r="B35" s="6" t="inlineStr">
+      <c r="B35" s="7" t="inlineStr">
         <is>
           <t>Compliance Monitoring and Safety Engineer</t>
         </is>
       </c>
-      <c r="C35" s="6" t="inlineStr">
+      <c r="C35" s="7" t="inlineStr">
         <is>
           <t>MNG Airlines</t>
         </is>
       </c>
-      <c r="D35" s="6" t="inlineStr">
+      <c r="D35" s="7" t="inlineStr">
         <is>
           <t>Istanbul, Türkiye</t>
         </is>
       </c>
-      <c r="E35" s="6" t="inlineStr">
+      <c r="E35" s="4" t="inlineStr">
+        <is>
+          <t>Türkiye</t>
+        </is>
+      </c>
+      <c r="F35" s="7" t="inlineStr">
         <is>
           <t>On-site</t>
         </is>
       </c>
-      <c r="F35" s="4" t="n">
+      <c r="G35" s="5" t="n">
         <v>46239</v>
       </c>
-      <c r="G35" s="6" t="inlineStr">
-        <is>
-          <t>Beklemede</t>
-        </is>
-      </c>
-      <c r="H35" s="6" t="inlineStr"/>
-      <c r="I35" s="6" t="inlineStr"/>
+      <c r="H35" s="7" t="inlineStr">
+        <is>
+          <t>Beklemede</t>
+        </is>
+      </c>
+      <c r="I35" s="7" t="inlineStr"/>
+      <c r="J35" s="7" t="inlineStr"/>
     </row>
     <row r="36">
       <c r="A36" s="2" t="n">
@@ -1765,56 +1949,66 @@
           <t>Eindhoven Area</t>
         </is>
       </c>
-      <c r="E36" s="3" t="inlineStr">
+      <c r="E36" s="4" t="inlineStr">
+        <is>
+          <t>Hollanda</t>
+        </is>
+      </c>
+      <c r="F36" s="3" t="inlineStr">
         <is>
           <t>Hybrid</t>
         </is>
       </c>
-      <c r="F36" s="4" t="n">
+      <c r="G36" s="5" t="n">
         <v>46239</v>
       </c>
-      <c r="G36" s="7" t="inlineStr">
+      <c r="H36" s="8" t="inlineStr">
         <is>
           <t>No longer accepting applications</t>
         </is>
       </c>
-      <c r="H36" s="3" t="inlineStr"/>
       <c r="I36" s="3" t="inlineStr"/>
+      <c r="J36" s="3" t="inlineStr"/>
     </row>
     <row r="37">
-      <c r="A37" s="5" t="n">
+      <c r="A37" s="6" t="n">
         <v>36</v>
       </c>
-      <c r="B37" s="6" t="inlineStr">
+      <c r="B37" s="7" t="inlineStr">
         <is>
           <t>European Product Safety &amp; Compliance Specialist</t>
         </is>
       </c>
-      <c r="C37" s="6" t="inlineStr">
+      <c r="C37" s="7" t="inlineStr">
         <is>
           <t>Midea</t>
         </is>
       </c>
-      <c r="D37" s="6" t="inlineStr">
+      <c r="D37" s="7" t="inlineStr">
         <is>
           <t>Zaragoza</t>
         </is>
       </c>
-      <c r="E37" s="6" t="inlineStr">
+      <c r="E37" s="4" t="inlineStr">
+        <is>
+          <t>İspanya</t>
+        </is>
+      </c>
+      <c r="F37" s="7" t="inlineStr">
         <is>
           <t>On-site</t>
         </is>
       </c>
-      <c r="F37" s="4" t="n">
+      <c r="G37" s="5" t="n">
         <v>46239</v>
       </c>
-      <c r="G37" s="6" t="inlineStr">
-        <is>
-          <t>Beklemede</t>
-        </is>
-      </c>
-      <c r="H37" s="6" t="inlineStr"/>
-      <c r="I37" s="6" t="inlineStr"/>
+      <c r="H37" s="7" t="inlineStr">
+        <is>
+          <t>Beklemede</t>
+        </is>
+      </c>
+      <c r="I37" s="7" t="inlineStr"/>
+      <c r="J37" s="7" t="inlineStr"/>
     </row>
     <row r="38">
       <c r="A38" s="2" t="n">
@@ -1835,56 +2029,66 @@
           <t>Dubai, United Arab Emirates</t>
         </is>
       </c>
-      <c r="E38" s="3" t="inlineStr">
+      <c r="E38" s="4" t="inlineStr">
+        <is>
+          <t>Birleşik Arap Emirlikleri</t>
+        </is>
+      </c>
+      <c r="F38" s="3" t="inlineStr">
         <is>
           <t>On-site</t>
         </is>
       </c>
-      <c r="F38" s="4" t="n">
+      <c r="G38" s="5" t="n">
         <v>46239</v>
       </c>
-      <c r="G38" s="7" t="inlineStr">
+      <c r="H38" s="8" t="inlineStr">
         <is>
           <t>No longer accepting applications</t>
         </is>
       </c>
-      <c r="H38" s="3" t="inlineStr"/>
       <c r="I38" s="3" t="inlineStr"/>
+      <c r="J38" s="3" t="inlineStr"/>
     </row>
     <row r="39">
-      <c r="A39" s="5" t="n">
+      <c r="A39" s="6" t="n">
         <v>38</v>
       </c>
-      <c r="B39" s="6" t="inlineStr">
+      <c r="B39" s="7" t="inlineStr">
         <is>
           <t>Product Safety &amp; Certifications Engineer / Field Evaluation Engineer</t>
         </is>
       </c>
-      <c r="C39" s="6" t="inlineStr">
+      <c r="C39" s="7" t="inlineStr">
         <is>
           <t>Product Safety Consulting</t>
         </is>
       </c>
-      <c r="D39" s="6" t="inlineStr">
+      <c r="D39" s="7" t="inlineStr">
         <is>
           <t>Bensenville, IL</t>
         </is>
       </c>
-      <c r="E39" s="6" t="inlineStr">
+      <c r="E39" s="4" t="inlineStr">
+        <is>
+          <t>ABD</t>
+        </is>
+      </c>
+      <c r="F39" s="7" t="inlineStr">
         <is>
           <t>Hybrid</t>
         </is>
       </c>
-      <c r="F39" s="4" t="n">
+      <c r="G39" s="5" t="n">
         <v>46239</v>
       </c>
-      <c r="G39" s="6" t="inlineStr">
-        <is>
-          <t>Beklemede</t>
-        </is>
-      </c>
-      <c r="H39" s="6" t="inlineStr"/>
-      <c r="I39" s="6" t="inlineStr"/>
+      <c r="H39" s="7" t="inlineStr">
+        <is>
+          <t>Beklemede</t>
+        </is>
+      </c>
+      <c r="I39" s="7" t="inlineStr"/>
+      <c r="J39" s="7" t="inlineStr"/>
     </row>
     <row r="40">
       <c r="A40" s="2" t="n">
@@ -1905,59 +2109,69 @@
           <t>Greater Freiburg Area</t>
         </is>
       </c>
-      <c r="E40" s="3" t="inlineStr">
+      <c r="E40" s="4" t="inlineStr">
+        <is>
+          <t>Almanya</t>
+        </is>
+      </c>
+      <c r="F40" s="3" t="inlineStr">
         <is>
           <t>Hybrid</t>
         </is>
       </c>
-      <c r="F40" s="4" t="n">
+      <c r="G40" s="5" t="n">
         <v>46239</v>
       </c>
-      <c r="G40" s="3" t="inlineStr">
-        <is>
-          <t>Beklemede</t>
-        </is>
-      </c>
-      <c r="H40" s="3" t="inlineStr"/>
+      <c r="H40" s="3" t="inlineStr">
+        <is>
+          <t>Beklemede</t>
+        </is>
+      </c>
       <c r="I40" s="3" t="inlineStr"/>
+      <c r="J40" s="3" t="inlineStr"/>
     </row>
     <row r="41">
-      <c r="A41" s="5" t="n">
+      <c r="A41" s="6" t="n">
         <v>40</v>
       </c>
-      <c r="B41" s="6" t="inlineStr">
+      <c r="B41" s="7" t="inlineStr">
         <is>
           <t>Compliance Specialist</t>
         </is>
       </c>
-      <c r="C41" s="6" t="inlineStr">
+      <c r="C41" s="7" t="inlineStr">
         <is>
           <t>LHH</t>
         </is>
       </c>
-      <c r="D41" s="6" t="inlineStr">
+      <c r="D41" s="7" t="inlineStr">
         <is>
           <t>Chicago, IL</t>
         </is>
       </c>
-      <c r="E41" s="6" t="inlineStr">
+      <c r="E41" s="4" t="inlineStr">
+        <is>
+          <t>ABD</t>
+        </is>
+      </c>
+      <c r="F41" s="7" t="inlineStr">
         <is>
           <t>Hybrid</t>
         </is>
       </c>
-      <c r="F41" s="4" t="n">
+      <c r="G41" s="5" t="n">
         <v>46232</v>
       </c>
-      <c r="G41" s="6" t="inlineStr">
-        <is>
-          <t>Beklemede</t>
-        </is>
-      </c>
-      <c r="H41" s="6" t="inlineStr"/>
-      <c r="I41" s="6" t="inlineStr"/>
+      <c r="H41" s="7" t="inlineStr">
+        <is>
+          <t>Beklemede</t>
+        </is>
+      </c>
+      <c r="I41" s="7" t="inlineStr"/>
+      <c r="J41" s="7" t="inlineStr"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:I41"/>
+  <autoFilter ref="A1:J41"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -1968,7 +2182,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B16"/>
+  <dimension ref="A1:B30"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="40" customWidth="1" min="1" max="1"/>
@@ -1976,7 +2190,7 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="8" t="inlineStr">
+      <c r="A1" s="9" t="inlineStr">
         <is>
           <t>Başvuru Takip Özeti</t>
         </is>
@@ -2018,7 +2232,7 @@
           <t>Referans tarih (bugün)</t>
         </is>
       </c>
-      <c r="B6" s="9" t="n">
+      <c r="B6" s="10" t="n">
         <v>46246</v>
       </c>
     </row>
@@ -2051,19 +2265,19 @@
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="10" t="inlineStr">
-        <is>
-          <t>Şirkete göre başvuru sayısı</t>
+      <c r="A13" s="11" t="inlineStr">
+        <is>
+          <t>Ülkeye göre başvuru sayısı</t>
         </is>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="10" t="inlineStr">
-        <is>
-          <t>Şirket</t>
-        </is>
-      </c>
-      <c r="B14" s="10" t="inlineStr">
+      <c r="A14" s="11" t="inlineStr">
+        <is>
+          <t>Ülke</t>
+        </is>
+      </c>
+      <c r="B14" s="11" t="inlineStr">
         <is>
           <t>Adet</t>
         </is>
@@ -2072,20 +2286,139 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Platform Recruitment</t>
+          <t>Birleşik Krallık</t>
         </is>
       </c>
       <c r="B15" t="n">
-        <v>2</v>
+        <v>24</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
+          <t>Türkiye</t>
+        </is>
+      </c>
+      <c r="B16" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>Hollanda</t>
+        </is>
+      </c>
+      <c r="B17" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>Almanya</t>
+        </is>
+      </c>
+      <c r="B18" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>ABD</t>
+        </is>
+      </c>
+      <c r="B19" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>İsveç</t>
+        </is>
+      </c>
+      <c r="B20" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>Belçika</t>
+        </is>
+      </c>
+      <c r="B21" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>İtalya</t>
+        </is>
+      </c>
+      <c r="B22" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>İspanya</t>
+        </is>
+      </c>
+      <c r="B23" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>Birleşik Arap Emirlikleri</t>
+        </is>
+      </c>
+      <c r="B24" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="11" t="inlineStr">
+        <is>
+          <t>Şirkete göre birden fazla başvuru</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="11" t="inlineStr">
+        <is>
+          <t>Şirket</t>
+        </is>
+      </c>
+      <c r="B28" s="11" t="inlineStr">
+        <is>
+          <t>Adet</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>Platform Recruitment</t>
+        </is>
+      </c>
+      <c r="B29" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
           <t>Solutions Driven</t>
         </is>
       </c>
-      <c r="B16" t="n">
+      <c r="B30" t="n">
         <v>2</v>
       </c>
     </row>

</xml_diff>